<commit_message>
feat: implement executive brief export pipeline, frontend components, and comprehensive audit reports
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -460,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-09-30T18:18:47.914Z</v>
+        <v>2026-10-01T06:55:30.021Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-09-30T18:18:47.915Z</v>
+        <v>2026-10-01T06:55:30.021Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add executive brief feature with frontend components, backend services, tests, and validation reports
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -460,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-01T06:55:30.021Z</v>
+        <v>2026-10-01T17:19:51.907Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-01T06:55:30.021Z</v>
+        <v>2026-10-01T17:19:51.907Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add subscription management, executive brief export services, and related UI components with test suites
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -460,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-02T08:27:34.504Z</v>
+        <v>2026-10-03T03:51:07.390Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-02T08:27:34.504Z</v>
+        <v>2026-10-03T03:51:07.390Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add enterprise evidence workbook generation, analysis orchestration, and audit reporting capabilities
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -460,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-03T16:08:12.309Z</v>
+        <v>2026-10-04T11:49:48.769Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-03T16:08:12.309Z</v>
+        <v>2026-10-04T11:49:48.770Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add enterprise evidence workbook generation, analysis orchestration, and audit reporting capabilities (#19)
Co-authored-by: srini2search-source <srini2search-source@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -460,7 +460,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-03T16:08:12.309Z</v>
+        <v>2026-10-04T11:49:48.769Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-03T16:08:12.309Z</v>
+        <v>2026-10-04T11:49:48.770Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Module 1 and Module 2 audit reports, backend services, and frontend orchestration components
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -460,7 +461,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-04T11:49:48.769Z</v>
+        <v>2026-10-06T10:38:30.071Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +493,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-04T11:49:48.770Z</v>
+        <v>2026-10-06T10:38:30.071Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Module 1 and Module 2 audit reports, backend services, and frontend orchestration components (#21)
Co-authored-by: srini2search-source <srini2search-source@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
+++ b/backend/MODULE_1_EXCEPTION_LEDGER.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -460,7 +461,7 @@
         <v>Documented PERIOD_SCOPE_MISMATCH in UI metadata and certification report</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-04T11:49:48.769Z</v>
+        <v>2026-10-06T10:38:30.071Z</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +493,7 @@
         <v>Unified regex to accept both alphanumeric and numeric SKUs; sample SKU aligned with unique items count</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-04T11:49:48.770Z</v>
+        <v>2026-10-06T10:38:30.071Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>